<commit_message>
Implement control mode architecture
</commit_message>
<xml_diff>
--- a/Dev/Tools/Servo calibration table.xlsx
+++ b/Dev/Tools/Servo calibration table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Quadro_Rob\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Quadro_Rob\Dev\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F5BFEA-554C-47BE-A7B0-B634C8562028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1198E728-6BDA-499F-8CB3-CE4744800D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2373D705-BA93-4439-8471-DD12D1F77279}"/>
   </bookViews>
@@ -812,10 +812,10 @@
         <v>265</v>
       </c>
       <c r="H7" s="17">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="I7" s="17">
-        <v>410</v>
+        <v>376</v>
       </c>
       <c r="J7" s="17"/>
       <c r="K7" s="17"/>

</xml_diff>

<commit_message>
Reorganize NovaQ connect project
</commit_message>
<xml_diff>
--- a/Dev/Tools/Servo calibration table.xlsx
+++ b/Dev/Tools/Servo calibration table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Quadro_Rob\Dev\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1198E728-6BDA-499F-8CB3-CE4744800D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D90AE06-3F1C-47BC-9491-F316A27E5CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2373D705-BA93-4439-8471-DD12D1F77279}"/>
+    <workbookView xWindow="3552" yWindow="3360" windowWidth="15468" windowHeight="8880" xr2:uid="{2373D705-BA93-4439-8471-DD12D1F77279}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -762,10 +762,10 @@
         <v>280</v>
       </c>
       <c r="H5" s="17">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="I5" s="17">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="J5" s="17"/>
       <c r="K5" s="17"/>
@@ -812,10 +812,10 @@
         <v>265</v>
       </c>
       <c r="H7" s="17">
-        <v>158</v>
+        <v>215</v>
       </c>
       <c r="I7" s="17">
-        <v>376</v>
+        <v>440</v>
       </c>
       <c r="J7" s="17"/>
       <c r="K7" s="17"/>
@@ -862,10 +862,10 @@
         <v>295</v>
       </c>
       <c r="H9" s="17">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="I9" s="17">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>

</xml_diff>